<commit_message>
Allow collisions becomes Colocate, in two versions (same instructor, different instructors)
Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-with-conflicts.xlsx
+++ b/apps/web/public/examples/example-with-conflicts.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="180">
   <si>
     <t>Term</t>
   </si>
@@ -73,6 +73,15 @@
     <t>CrossListings</t>
   </si>
   <si>
+    <t>CoreTag</t>
+  </si>
+  <si>
+    <t>SpecialTopic</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
     <t>FA</t>
   </si>
   <si>
@@ -121,6 +130,9 @@
     <t/>
   </si>
   <si>
+    <t>UGRAD</t>
+  </si>
+  <si>
     <t>B</t>
   </si>
   <si>
@@ -511,13 +523,13 @@
     <t>Export Date</t>
   </si>
   <si>
-    <t>2026-10-04</t>
+    <t>2026-10-06</t>
   </si>
   <si>
     <t>Export Time</t>
   </si>
   <si>
-    <t>21:03:16</t>
+    <t>13:27:37</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -925,7 +937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:U12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -944,9 +956,11 @@
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="40" customWidth="1"/>
     <col min="18" max="18" width="15" customWidth="1"/>
+    <col min="20" max="20" width="14" customWidth="1"/>
+    <col min="21" max="21" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1001,621 +1015,729 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="J2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="L2">
         <v>65</v>
       </c>
       <c r="M2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="N2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" t="s">
+        <v>36</v>
+      </c>
+      <c r="S2" t="s">
+        <v>36</v>
+      </c>
+      <c r="T2" t="s">
+        <v>36</v>
+      </c>
+      <c r="U2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" t="s">
         <v>29</v>
       </c>
-      <c r="O2" t="s">
+      <c r="K3" t="s">
         <v>30</v>
-      </c>
-      <c r="P2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>32</v>
-      </c>
-      <c r="R2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K3" t="s">
-        <v>27</v>
       </c>
       <c r="L3">
         <v>65</v>
       </c>
       <c r="M3" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>36</v>
+      </c>
+      <c r="R3" t="s">
+        <v>36</v>
+      </c>
+      <c r="S3" t="s">
+        <v>36</v>
+      </c>
+      <c r="T3" t="s">
+        <v>36</v>
+      </c>
+      <c r="U3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" t="s">
         <v>28</v>
       </c>
-      <c r="N3" t="s">
+      <c r="J4" t="s">
         <v>29</v>
       </c>
-      <c r="O3" t="s">
-        <v>30</v>
-      </c>
-      <c r="P3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>33</v>
-      </c>
-      <c r="R3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
-      </c>
       <c r="K4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="L4">
         <v>65</v>
       </c>
       <c r="M4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="N4" t="s">
+        <v>32</v>
+      </c>
+      <c r="O4" t="s">
+        <v>33</v>
+      </c>
+      <c r="P4" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>44</v>
+      </c>
+      <c r="R4" t="s">
+        <v>36</v>
+      </c>
+      <c r="S4" t="s">
+        <v>36</v>
+      </c>
+      <c r="T4" t="s">
+        <v>36</v>
+      </c>
+      <c r="U4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" t="s">
+        <v>47</v>
+      </c>
+      <c r="J5" t="s">
         <v>29</v>
       </c>
-      <c r="O4" t="s">
+      <c r="K5" t="s">
         <v>30</v>
-      </c>
-      <c r="P4" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>40</v>
-      </c>
-      <c r="R4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" t="s">
-        <v>26</v>
-      </c>
-      <c r="K5" t="s">
-        <v>27</v>
       </c>
       <c r="L5">
         <v>65</v>
       </c>
       <c r="M5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="N5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="O5" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>50</v>
+      </c>
+      <c r="R5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S5" t="s">
+        <v>36</v>
+      </c>
+      <c r="T5" t="s">
+        <v>36</v>
+      </c>
+      <c r="U5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J6" t="s">
+        <v>29</v>
+      </c>
+      <c r="K6" t="s">
         <v>30</v>
-      </c>
-      <c r="P5" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>46</v>
-      </c>
-      <c r="R5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" t="s">
-        <v>49</v>
-      </c>
-      <c r="I6" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" t="s">
-        <v>26</v>
-      </c>
-      <c r="K6" t="s">
-        <v>27</v>
       </c>
       <c r="L6">
         <v>100</v>
       </c>
       <c r="M6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="N6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="O6" t="s">
+        <v>33</v>
+      </c>
+      <c r="P6" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>56</v>
+      </c>
+      <c r="R6" t="s">
+        <v>36</v>
+      </c>
+      <c r="S6" t="s">
+        <v>36</v>
+      </c>
+      <c r="T6" t="s">
+        <v>36</v>
+      </c>
+      <c r="U6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" t="s">
+        <v>52</v>
+      </c>
+      <c r="H7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J7" t="s">
+        <v>29</v>
+      </c>
+      <c r="K7" t="s">
         <v>30</v>
-      </c>
-      <c r="P6" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>52</v>
-      </c>
-      <c r="R6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" t="s">
-        <v>48</v>
-      </c>
-      <c r="H7" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" t="s">
-        <v>26</v>
-      </c>
-      <c r="K7" t="s">
-        <v>27</v>
       </c>
       <c r="L7">
         <v>100</v>
       </c>
       <c r="M7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="N7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="O7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>62</v>
+      </c>
+      <c r="R7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S7" t="s">
+        <v>36</v>
+      </c>
+      <c r="T7" t="s">
+        <v>36</v>
+      </c>
+      <c r="U7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="s">
+        <v>64</v>
+      </c>
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" t="s">
         <v>30</v>
-      </c>
-      <c r="P7" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>58</v>
-      </c>
-      <c r="R7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" t="s">
-        <v>22</v>
-      </c>
-      <c r="F8" t="s">
-        <v>22</v>
-      </c>
-      <c r="G8" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" t="s">
-        <v>60</v>
-      </c>
-      <c r="I8" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" t="s">
-        <v>26</v>
-      </c>
-      <c r="K8" t="s">
-        <v>27</v>
       </c>
       <c r="L8">
         <v>65</v>
       </c>
       <c r="M8" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="N8" t="s">
+        <v>67</v>
+      </c>
+      <c r="O8" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>36</v>
+      </c>
+      <c r="R8" t="s">
+        <v>36</v>
+      </c>
+      <c r="S8" t="s">
+        <v>36</v>
+      </c>
+      <c r="T8" t="s">
+        <v>36</v>
+      </c>
+      <c r="U8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s">
         <v>63</v>
       </c>
-      <c r="O8" t="s">
+      <c r="C9" t="s">
+        <v>68</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" t="s">
+        <v>54</v>
+      </c>
+      <c r="J9" t="s">
+        <v>29</v>
+      </c>
+      <c r="K9" t="s">
         <v>30</v>
-      </c>
-      <c r="P8" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>33</v>
-      </c>
-      <c r="R8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9" t="s">
-        <v>22</v>
-      </c>
-      <c r="F9" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" t="s">
-        <v>49</v>
-      </c>
-      <c r="I9" t="s">
-        <v>50</v>
-      </c>
-      <c r="J9" t="s">
-        <v>26</v>
-      </c>
-      <c r="K9" t="s">
-        <v>27</v>
       </c>
       <c r="L9">
         <v>100</v>
       </c>
       <c r="M9" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="N9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="P9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="S9" t="s">
+        <v>36</v>
+      </c>
+      <c r="T9" t="s">
+        <v>36</v>
+      </c>
+      <c r="U9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="I10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="J10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="K10" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="L10">
         <v>100</v>
       </c>
       <c r="M10" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="N10" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="O10" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>36</v>
+      </c>
+      <c r="R10" t="s">
+        <v>36</v>
+      </c>
+      <c r="S10" t="s">
+        <v>36</v>
+      </c>
+      <c r="T10" t="s">
+        <v>36</v>
+      </c>
+      <c r="U10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>73</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
+        <v>64</v>
+      </c>
+      <c r="I11" t="s">
+        <v>59</v>
+      </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" t="s">
         <v>30</v>
-      </c>
-      <c r="P10" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>33</v>
-      </c>
-      <c r="R10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" t="s">
-        <v>69</v>
-      </c>
-      <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
-      </c>
-      <c r="F11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" t="s">
-        <v>60</v>
-      </c>
-      <c r="I11" t="s">
-        <v>55</v>
-      </c>
-      <c r="J11" t="s">
-        <v>26</v>
-      </c>
-      <c r="K11" t="s">
-        <v>27</v>
       </c>
       <c r="L11">
         <v>65</v>
       </c>
       <c r="M11" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N11" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="O11" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" t="s">
+        <v>34</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>76</v>
+      </c>
+      <c r="R11" t="s">
+        <v>36</v>
+      </c>
+      <c r="S11" t="s">
+        <v>36</v>
+      </c>
+      <c r="T11" t="s">
+        <v>36</v>
+      </c>
+      <c r="U11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" t="s">
+        <v>79</v>
+      </c>
+      <c r="I12" t="s">
+        <v>80</v>
+      </c>
+      <c r="J12" t="s">
+        <v>29</v>
+      </c>
+      <c r="K12" t="s">
         <v>30</v>
-      </c>
-      <c r="P11" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>72</v>
-      </c>
-      <c r="R11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>18</v>
-      </c>
-      <c r="B12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12" t="s">
-        <v>22</v>
-      </c>
-      <c r="F12" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" t="s">
-        <v>48</v>
-      </c>
-      <c r="H12" t="s">
-        <v>75</v>
-      </c>
-      <c r="I12" t="s">
-        <v>76</v>
-      </c>
-      <c r="J12" t="s">
-        <v>26</v>
-      </c>
-      <c r="K12" t="s">
-        <v>27</v>
       </c>
       <c r="L12">
         <v>100</v>
       </c>
       <c r="M12" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="N12" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="O12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="P12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R12" t="s">
-        <v>33</v>
+        <v>36</v>
+      </c>
+      <c r="S12" t="s">
+        <v>36</v>
+      </c>
+      <c r="T12" t="s">
+        <v>36</v>
+      </c>
+      <c r="U12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1626,7 +1748,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
@@ -1651,17 +1773,18 @@
     <col min="22" max="22" width="40" customWidth="1"/>
     <col min="23" max="23" width="12" customWidth="1"/>
     <col min="24" max="24" width="17" customWidth="1"/>
+    <col min="26" max="26" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1685,22 +1808,22 @@
         <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>12</v>
@@ -1709,10 +1832,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>15</v>
@@ -1721,39 +1844,45 @@
         <v>16</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J2">
         <v>4</v>
@@ -1762,72 +1891,78 @@
         <v>4</v>
       </c>
       <c r="L2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="O2">
         <v>65</v>
       </c>
       <c r="P2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="Q2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="R2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V2" t="s">
+        <v>35</v>
+      </c>
+      <c r="W2" t="s">
+        <v>36</v>
+      </c>
+      <c r="X2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H3" t="s">
+        <v>38</v>
+      </c>
+      <c r="I3" t="s">
         <v>32</v>
-      </c>
-      <c r="W2" t="s">
-        <v>33</v>
-      </c>
-      <c r="X2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>93</v>
-      </c>
-      <c r="B3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>29</v>
       </c>
       <c r="J3">
         <v>4</v>
@@ -1836,72 +1971,78 @@
         <v>4</v>
       </c>
       <c r="L3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="O3">
         <v>65</v>
       </c>
       <c r="P3" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="Q3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="R3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="W3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="H4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J4">
         <v>4</v>
@@ -1910,72 +2051,78 @@
         <v>4</v>
       </c>
       <c r="L4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="N4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O4">
         <v>100</v>
       </c>
       <c r="P4" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="Q4" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="R4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V4" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="W4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H5" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -1984,72 +2131,78 @@
         <v>4</v>
       </c>
       <c r="L5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="N5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O5">
         <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="Q5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="R5" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="W5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X5" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -2058,72 +2211,78 @@
         <v>4</v>
       </c>
       <c r="L6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M6" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="O6">
         <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="Q6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="R6" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="W6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F7" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I7" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J7">
         <v>4</v>
@@ -2132,72 +2291,78 @@
         <v>4</v>
       </c>
       <c r="L7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M7" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="N7" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="O7">
         <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="R7" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V7" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="W7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="H8" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I8" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -2206,72 +2371,78 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M8" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="N8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="O8">
         <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="Q8" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="R8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="W8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y8" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I9" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="J9">
         <v>4</v>
@@ -2280,72 +2451,78 @@
         <v>4</v>
       </c>
       <c r="L9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M9" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N9" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="O9">
         <v>65</v>
       </c>
       <c r="P9" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="Q9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="R9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V9" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="W9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X9" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H10" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="J10">
         <v>4</v>
@@ -2354,72 +2531,78 @@
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M10" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N10" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="O10">
         <v>65</v>
       </c>
       <c r="P10" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="Q10" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="R10" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="W10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+      <c r="Y10" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J11">
         <v>4</v>
@@ -2428,72 +2611,78 @@
         <v>4</v>
       </c>
       <c r="L11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M11" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="N11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="O11">
         <v>65</v>
       </c>
       <c r="P11" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="Q11" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="R11" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V11" t="s">
+        <v>44</v>
+      </c>
+      <c r="W11" t="s">
+        <v>36</v>
+      </c>
+      <c r="X11" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" t="s">
         <v>40</v>
       </c>
-      <c r="W11" t="s">
-        <v>33</v>
-      </c>
-      <c r="X11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>107</v>
-      </c>
-      <c r="B12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D12" t="s">
-        <v>36</v>
-      </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H12" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J12">
         <v>4</v>
@@ -2502,43 +2691,49 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M12" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="N12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="O12">
         <v>100</v>
       </c>
       <c r="P12" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="Q12" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="R12" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="S12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="U12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="V12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="W12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="X12" t="s">
-        <v>33</v>
+        <v>36</v>
+      </c>
+      <c r="Y12" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z12" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2559,7 +2754,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2586,19 +2781,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
@@ -2635,61 +2830,61 @@
   <sheetData>
     <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="T1" s="1" t="s">
         <v>16</v>
@@ -2697,188 +2892,188 @@
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="O2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="P2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="Q2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="O3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="P3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="Q3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="J4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="K4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="L4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="M4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="N4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="P4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="Q4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="T4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2900,122 +3095,122 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3023,19 +3218,19 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -3043,19 +3238,19 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -3063,19 +3258,19 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C9" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -3083,33 +3278,33 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C10" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -3120,16 +3315,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B12" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C12" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -3140,16 +3335,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B13" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C13" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E13">
         <v>9</v>
@@ -3160,16 +3355,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -3180,16 +3375,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E15">
         <v>5</v>
@@ -3200,16 +3395,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B16" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="C16" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E16">
         <v>9</v>
@@ -3220,16 +3415,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B17" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C17" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E17">
         <v>13</v>
@@ -3240,16 +3435,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C18" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D18" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -3275,90 +3470,90 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B8" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New example: Merging schedules, with a cohort planning rule that fails when merged
Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-with-conflicts.xlsx
+++ b/apps/web/public/examples/example-with-conflicts.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="184">
   <si>
     <t>Term</t>
   </si>
@@ -82,6 +82,9 @@
     <t>Level</t>
   </si>
   <si>
+    <t>Colocations</t>
+  </si>
+  <si>
     <t>FA</t>
   </si>
   <si>
@@ -409,6 +412,15 @@
     <t>Meets</t>
   </si>
   <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
     <t>AMUS major, year 2</t>
   </si>
   <si>
@@ -418,6 +430,9 @@
     <t>AMUS 228</t>
   </si>
   <si>
+    <t>Yes</t>
+  </si>
+  <si>
     <t>A student in this cohort should be able to take all three courses. AMUS 228 and BHAV 212 each have one section and meet at the same time</t>
   </si>
   <si>
@@ -523,13 +538,13 @@
     <t>Export Date</t>
   </si>
   <si>
-    <t>2026-10-06</t>
+    <t>2026-10-07</t>
   </si>
   <si>
     <t>Export Time</t>
   </si>
   <si>
-    <t>13:27:37</t>
+    <t>08:51:36</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -545,9 +560,6 @@
   </si>
   <si>
     <t>Time Stamp In File Name</t>
-  </si>
-  <si>
-    <t>Yes</t>
   </si>
   <si>
     <t>Default Department</t>
@@ -937,7 +949,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U12"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -958,9 +970,10 @@
     <col min="18" max="18" width="15" customWidth="1"/>
     <col min="20" max="20" width="14" customWidth="1"/>
     <col min="21" max="21" width="7" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1024,719 +1037,755 @@
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L2">
         <v>65</v>
       </c>
       <c r="M2" t="s">
+        <v>32</v>
+      </c>
+      <c r="N2" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P2" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>36</v>
+      </c>
+      <c r="R2" t="s">
+        <v>37</v>
+      </c>
+      <c r="S2" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" t="s">
+        <v>37</v>
+      </c>
+      <c r="U2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+      <c r="J3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" t="s">
         <v>31</v>
-      </c>
-      <c r="N2" t="s">
-        <v>32</v>
-      </c>
-      <c r="O2" t="s">
-        <v>33</v>
-      </c>
-      <c r="P2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>35</v>
-      </c>
-      <c r="R2" t="s">
-        <v>36</v>
-      </c>
-      <c r="S2" t="s">
-        <v>36</v>
-      </c>
-      <c r="T2" t="s">
-        <v>36</v>
-      </c>
-      <c r="U2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" t="s">
-        <v>39</v>
-      </c>
-      <c r="J3" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" t="s">
-        <v>30</v>
       </c>
       <c r="L3">
         <v>65</v>
       </c>
       <c r="M3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L4">
         <v>65</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="N4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="R4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L5">
         <v>65</v>
       </c>
       <c r="M5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="R5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L6">
         <v>100</v>
       </c>
       <c r="M6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="R6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L7">
         <v>100</v>
       </c>
       <c r="M7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="O7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="R7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H8" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L8">
         <v>65</v>
       </c>
       <c r="M8" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="N8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="O8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U8" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L9">
         <v>100</v>
       </c>
       <c r="M9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H10" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L10">
         <v>100</v>
       </c>
       <c r="M10" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="N10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="O10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U10" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L11">
         <v>65</v>
       </c>
       <c r="M11" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N11" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="R11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+        <v>38</v>
+      </c>
+      <c r="V11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H12" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K12" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L12">
         <v>100</v>
       </c>
       <c r="M12" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="N12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="O12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U12" t="s">
+        <v>38</v>
+      </c>
+      <c r="V12" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1778,13 +1827,13 @@
   <sheetData>
     <row r="1" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -1808,22 +1857,22 @@
         <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>12</v>
@@ -1832,10 +1881,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>15</v>
@@ -1844,10 +1893,10 @@
         <v>16</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>18</v>
@@ -1858,31 +1907,31 @@
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J2">
         <v>4</v>
@@ -1891,78 +1940,78 @@
         <v>4</v>
       </c>
       <c r="L2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O2">
         <v>65</v>
       </c>
       <c r="P2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" t="s">
+        <v>37</v>
+      </c>
+      <c r="U2" t="s">
+        <v>35</v>
+      </c>
+      <c r="V2" t="s">
         <v>36</v>
       </c>
-      <c r="T2" t="s">
-        <v>36</v>
-      </c>
-      <c r="U2" t="s">
-        <v>34</v>
-      </c>
-      <c r="V2" t="s">
-        <v>35</v>
-      </c>
       <c r="W2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J3">
         <v>4</v>
@@ -1971,78 +2020,78 @@
         <v>4</v>
       </c>
       <c r="L3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O3">
         <v>65</v>
       </c>
       <c r="P3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J4">
         <v>4</v>
@@ -2051,78 +2100,78 @@
         <v>4</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O4">
         <v>100</v>
       </c>
       <c r="P4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="R4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="W4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -2131,78 +2180,78 @@
         <v>4</v>
       </c>
       <c r="L5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O5">
         <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="R5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -2211,78 +2260,78 @@
         <v>4</v>
       </c>
       <c r="L6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="O6">
         <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="Q6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="W6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J7">
         <v>4</v>
@@ -2291,78 +2340,78 @@
         <v>4</v>
       </c>
       <c r="L7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="O7">
         <v>100</v>
       </c>
       <c r="P7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="R7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="W7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -2371,78 +2420,78 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="O8">
         <v>100</v>
       </c>
       <c r="P8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="Q8" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="R8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J9">
         <v>4</v>
@@ -2451,78 +2500,78 @@
         <v>4</v>
       </c>
       <c r="L9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O9">
         <v>65</v>
       </c>
       <c r="P9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="Q9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="R9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="W9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I10" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="J10">
         <v>4</v>
@@ -2531,78 +2580,78 @@
         <v>4</v>
       </c>
       <c r="L10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N10" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O10">
         <v>65</v>
       </c>
       <c r="P10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q10" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J11">
         <v>4</v>
@@ -2611,78 +2660,78 @@
         <v>4</v>
       </c>
       <c r="L11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N11" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="O11">
         <v>65</v>
       </c>
       <c r="P11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="Q11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U11" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="W11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H12" t="s">
+        <v>25</v>
+      </c>
+      <c r="I12" t="s">
         <v>71</v>
-      </c>
-      <c r="H12" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" t="s">
-        <v>70</v>
       </c>
       <c r="J12">
         <v>4</v>
@@ -2691,49 +2740,49 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="N12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="O12">
         <v>100</v>
       </c>
       <c r="P12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="Q12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R12" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="S12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="U12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="W12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Y12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Z12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2754,7 +2803,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2781,19 +2830,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
@@ -2807,7 +2856,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2825,255 +2874,293 @@
     <col min="17" max="17" width="4" customWidth="1"/>
     <col min="18" max="18" width="8" customWidth="1"/>
     <col min="19" max="19" width="7" customWidth="1"/>
-    <col min="20" max="20" width="40" customWidth="1"/>
+    <col min="21" max="21" width="10" customWidth="1"/>
+    <col min="22" max="22" width="8" customWidth="1"/>
+    <col min="23" max="23" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+      <c r="U2" t="s">
+        <v>37</v>
+      </c>
+      <c r="V2" t="s">
+        <v>137</v>
+      </c>
+      <c r="W2" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D3" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>37</v>
+      </c>
+      <c r="G3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I3" t="s">
+        <v>37</v>
+      </c>
+      <c r="J3" t="s">
+        <v>37</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M3" t="s">
+        <v>37</v>
+      </c>
+      <c r="N3" t="s">
+        <v>37</v>
+      </c>
+      <c r="O3" t="s">
+        <v>37</v>
+      </c>
+      <c r="P3" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>37</v>
+      </c>
+      <c r="R3" t="s">
+        <v>37</v>
+      </c>
+      <c r="S3" t="s">
+        <v>37</v>
+      </c>
+      <c r="T3" t="s">
+        <v>37</v>
+      </c>
+      <c r="U3" t="s">
+        <v>37</v>
+      </c>
+      <c r="V3" t="s">
+        <v>137</v>
+      </c>
+      <c r="W3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>134</v>
       </c>
-      <c r="D3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" t="s">
-        <v>36</v>
-      </c>
-      <c r="F3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J3" t="s">
-        <v>36</v>
-      </c>
-      <c r="K3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" t="s">
-        <v>36</v>
-      </c>
-      <c r="M3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N3" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3" t="s">
-        <v>36</v>
-      </c>
-      <c r="P3" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" t="s">
-        <v>36</v>
-      </c>
-      <c r="S3" t="s">
-        <v>36</v>
-      </c>
-      <c r="T3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>130</v>
-      </c>
       <c r="B4" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="K4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="N4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="O4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="P4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="T4" t="s">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="U4" t="s">
+        <v>37</v>
+      </c>
+      <c r="V4" t="s">
+        <v>137</v>
+      </c>
+      <c r="W4" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -3095,122 +3182,122 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B6" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3218,19 +3305,19 @@
         <v>0</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -3238,19 +3325,19 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C8" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -3258,19 +3345,19 @@
         <v>0</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -3278,33 +3365,33 @@
         <v>0</v>
       </c>
       <c r="B10" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C10" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C11" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -3315,16 +3402,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B12" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C12" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -3335,16 +3422,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B13" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C13" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E13">
         <v>9</v>
@@ -3355,16 +3442,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -3375,16 +3462,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E15">
         <v>5</v>
@@ -3395,16 +3482,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C16" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E16">
         <v>9</v>
@@ -3415,16 +3502,16 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B17" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C17" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E17">
         <v>13</v>
@@ -3435,16 +3522,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>157</v>
+      </c>
+      <c r="B18" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" t="s">
+        <v>169</v>
+      </c>
+      <c r="D18" t="s">
         <v>152</v>
-      </c>
-      <c r="B18" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D18" t="s">
-        <v>147</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -3470,90 +3557,90 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B8" t="s">
-        <v>176</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>